<commit_message>
Refactor admin portal and modularize frontend
</commit_message>
<xml_diff>
--- a/xa.xlsx
+++ b/xa.xlsx
@@ -8,17 +8,26 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Admin\Desktop\he_thong_bao_cao\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2FA92682-D8C4-4B52-854D-7C06FA7AB494}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{152820D0-4E15-4833-9B4C-44468DB1D148}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="4725" yWindow="0" windowWidth="15870" windowHeight="10905" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="162913"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
+    </ext>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+      </xcalcf:calcFeatures>
     </ext>
   </extLst>
 </workbook>
@@ -1011,7 +1020,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
@@ -1035,6 +1044,7 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1315,15 +1325,16 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:C154"/>
+  <dimension ref="A1:F154"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="5.85546875" customWidth="1"/>
     <col min="2" max="2" width="13.28515625" customWidth="1"/>
     <col min="3" max="3" width="14.85546875" customWidth="1"/>
+    <col min="7" max="7" width="32" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:6" ht="16.5" x14ac:dyDescent="0.25">
       <c r="A1" s="8" t="s">
         <v>308</v>
       </c>
@@ -1334,7 +1345,7 @@
         <v>305</v>
       </c>
     </row>
-    <row r="2" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:6" ht="16.5" x14ac:dyDescent="0.25">
       <c r="A2" s="7">
         <v>1</v>
       </c>
@@ -1344,8 +1355,11 @@
       <c r="C2" s="3" t="s">
         <v>152</v>
       </c>
-    </row>
-    <row r="3" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="D2" s="9"/>
+      <c r="E2" s="9"/>
+      <c r="F2" s="9"/>
+    </row>
+    <row r="3" spans="1:6" ht="16.5" x14ac:dyDescent="0.25">
       <c r="A3" s="7">
         <v>2</v>
       </c>
@@ -1355,8 +1369,11 @@
       <c r="C3" s="3" t="s">
         <v>153</v>
       </c>
-    </row>
-    <row r="4" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="D3" s="9"/>
+      <c r="E3" s="9"/>
+      <c r="F3" s="9"/>
+    </row>
+    <row r="4" spans="1:6" ht="16.5" x14ac:dyDescent="0.25">
       <c r="A4" s="7">
         <v>3</v>
       </c>
@@ -1366,8 +1383,11 @@
       <c r="C4" s="3" t="s">
         <v>154</v>
       </c>
-    </row>
-    <row r="5" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="D4" s="9"/>
+      <c r="E4" s="9"/>
+      <c r="F4" s="9"/>
+    </row>
+    <row r="5" spans="1:6" ht="16.5" x14ac:dyDescent="0.25">
       <c r="A5" s="7">
         <v>4</v>
       </c>
@@ -1377,8 +1397,11 @@
       <c r="C5" s="3" t="s">
         <v>155</v>
       </c>
-    </row>
-    <row r="6" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="D5" s="9"/>
+      <c r="E5" s="9"/>
+      <c r="F5" s="9"/>
+    </row>
+    <row r="6" spans="1:6" ht="16.5" x14ac:dyDescent="0.25">
       <c r="A6" s="7">
         <v>5</v>
       </c>
@@ -1388,8 +1411,11 @@
       <c r="C6" s="3" t="s">
         <v>156</v>
       </c>
-    </row>
-    <row r="7" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="D6" s="9"/>
+      <c r="E6" s="9"/>
+      <c r="F6" s="9"/>
+    </row>
+    <row r="7" spans="1:6" ht="16.5" x14ac:dyDescent="0.25">
       <c r="A7" s="7">
         <v>6</v>
       </c>
@@ -1399,8 +1425,11 @@
       <c r="C7" s="3" t="s">
         <v>269</v>
       </c>
-    </row>
-    <row r="8" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="D7" s="9"/>
+      <c r="E7" s="9"/>
+      <c r="F7" s="9"/>
+    </row>
+    <row r="8" spans="1:6" ht="16.5" x14ac:dyDescent="0.25">
       <c r="A8" s="7">
         <v>7</v>
       </c>
@@ -1410,8 +1439,11 @@
       <c r="C8" s="3" t="s">
         <v>270</v>
       </c>
-    </row>
-    <row r="9" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="D8" s="9"/>
+      <c r="E8" s="9"/>
+      <c r="F8" s="9"/>
+    </row>
+    <row r="9" spans="1:6" ht="16.5" x14ac:dyDescent="0.25">
       <c r="A9" s="7">
         <v>8</v>
       </c>
@@ -1421,8 +1453,11 @@
       <c r="C9" s="3" t="s">
         <v>295</v>
       </c>
-    </row>
-    <row r="10" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="D9" s="9"/>
+      <c r="E9" s="9"/>
+      <c r="F9" s="9"/>
+    </row>
+    <row r="10" spans="1:6" ht="16.5" x14ac:dyDescent="0.25">
       <c r="A10" s="7">
         <v>9</v>
       </c>
@@ -1432,8 +1467,11 @@
       <c r="C10" s="3" t="s">
         <v>161</v>
       </c>
-    </row>
-    <row r="11" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="D10" s="9"/>
+      <c r="E10" s="9"/>
+      <c r="F10" s="9"/>
+    </row>
+    <row r="11" spans="1:6" ht="16.5" x14ac:dyDescent="0.25">
       <c r="A11" s="7">
         <v>10</v>
       </c>
@@ -1443,8 +1481,11 @@
       <c r="C11" s="3" t="s">
         <v>177</v>
       </c>
-    </row>
-    <row r="12" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="D11" s="9"/>
+      <c r="E11" s="9"/>
+      <c r="F11" s="9"/>
+    </row>
+    <row r="12" spans="1:6" ht="16.5" x14ac:dyDescent="0.25">
       <c r="A12" s="7">
         <v>11</v>
       </c>
@@ -1454,8 +1495,11 @@
       <c r="C12" s="3" t="s">
         <v>275</v>
       </c>
-    </row>
-    <row r="13" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="D12" s="9"/>
+      <c r="E12" s="9"/>
+      <c r="F12" s="9"/>
+    </row>
+    <row r="13" spans="1:6" ht="16.5" x14ac:dyDescent="0.25">
       <c r="A13" s="7">
         <v>12</v>
       </c>
@@ -1465,8 +1509,11 @@
       <c r="C13" s="3" t="s">
         <v>242</v>
       </c>
-    </row>
-    <row r="14" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="D13" s="9"/>
+      <c r="E13" s="9"/>
+      <c r="F13" s="9"/>
+    </row>
+    <row r="14" spans="1:6" ht="16.5" x14ac:dyDescent="0.25">
       <c r="A14" s="7">
         <v>13</v>
       </c>
@@ -1476,8 +1523,11 @@
       <c r="C14" s="3" t="s">
         <v>166</v>
       </c>
-    </row>
-    <row r="15" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="D14" s="9"/>
+      <c r="E14" s="9"/>
+      <c r="F14" s="9"/>
+    </row>
+    <row r="15" spans="1:6" ht="16.5" x14ac:dyDescent="0.25">
       <c r="A15" s="7">
         <v>14</v>
       </c>
@@ -1487,8 +1537,11 @@
       <c r="C15" s="3" t="s">
         <v>245</v>
       </c>
-    </row>
-    <row r="16" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="D15" s="9"/>
+      <c r="E15" s="9"/>
+      <c r="F15" s="9"/>
+    </row>
+    <row r="16" spans="1:6" ht="16.5" x14ac:dyDescent="0.25">
       <c r="A16" s="7">
         <v>15</v>
       </c>
@@ -1498,8 +1551,11 @@
       <c r="C16" s="3" t="s">
         <v>244</v>
       </c>
-    </row>
-    <row r="17" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="D16" s="9"/>
+      <c r="E16" s="9"/>
+      <c r="F16" s="9"/>
+    </row>
+    <row r="17" spans="1:6" ht="16.5" x14ac:dyDescent="0.25">
       <c r="A17" s="7">
         <v>16</v>
       </c>
@@ -1509,8 +1565,11 @@
       <c r="C17" s="3" t="s">
         <v>184</v>
       </c>
-    </row>
-    <row r="18" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="D17" s="9"/>
+      <c r="E17" s="9"/>
+      <c r="F17" s="9"/>
+    </row>
+    <row r="18" spans="1:6" ht="16.5" x14ac:dyDescent="0.25">
       <c r="A18" s="7">
         <v>17</v>
       </c>
@@ -1520,8 +1579,11 @@
       <c r="C18" s="3" t="s">
         <v>272</v>
       </c>
-    </row>
-    <row r="19" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="D18" s="9"/>
+      <c r="E18" s="9"/>
+      <c r="F18" s="9"/>
+    </row>
+    <row r="19" spans="1:6" ht="16.5" x14ac:dyDescent="0.25">
       <c r="A19" s="7">
         <v>18</v>
       </c>
@@ -1531,8 +1593,11 @@
       <c r="C19" s="3" t="s">
         <v>247</v>
       </c>
-    </row>
-    <row r="20" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="D19" s="9"/>
+      <c r="E19" s="9"/>
+      <c r="F19" s="9"/>
+    </row>
+    <row r="20" spans="1:6" ht="16.5" x14ac:dyDescent="0.25">
       <c r="A20" s="7">
         <v>19</v>
       </c>
@@ -1542,8 +1607,11 @@
       <c r="C20" s="3" t="s">
         <v>251</v>
       </c>
-    </row>
-    <row r="21" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="D20" s="9"/>
+      <c r="E20" s="9"/>
+      <c r="F20" s="9"/>
+    </row>
+    <row r="21" spans="1:6" ht="16.5" x14ac:dyDescent="0.25">
       <c r="A21" s="7">
         <v>20</v>
       </c>
@@ -1553,8 +1621,11 @@
       <c r="C21" s="3" t="s">
         <v>175</v>
       </c>
-    </row>
-    <row r="22" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="D21" s="9"/>
+      <c r="E21" s="9"/>
+      <c r="F21" s="9"/>
+    </row>
+    <row r="22" spans="1:6" ht="16.5" x14ac:dyDescent="0.25">
       <c r="A22" s="7">
         <v>21</v>
       </c>
@@ -1564,8 +1635,11 @@
       <c r="C22" s="3" t="s">
         <v>176</v>
       </c>
-    </row>
-    <row r="23" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="D22" s="9"/>
+      <c r="E22" s="9"/>
+      <c r="F22" s="9"/>
+    </row>
+    <row r="23" spans="1:6" ht="16.5" x14ac:dyDescent="0.25">
       <c r="A23" s="7">
         <v>22</v>
       </c>
@@ -1575,8 +1649,11 @@
       <c r="C23" s="3" t="s">
         <v>171</v>
       </c>
-    </row>
-    <row r="24" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="D23" s="9"/>
+      <c r="E23" s="9"/>
+      <c r="F23" s="9"/>
+    </row>
+    <row r="24" spans="1:6" ht="16.5" x14ac:dyDescent="0.25">
       <c r="A24" s="7">
         <v>23</v>
       </c>
@@ -1586,8 +1663,11 @@
       <c r="C24" s="3" t="s">
         <v>200</v>
       </c>
-    </row>
-    <row r="25" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="D24" s="9"/>
+      <c r="E24" s="9"/>
+      <c r="F24" s="9"/>
+    </row>
+    <row r="25" spans="1:6" ht="16.5" x14ac:dyDescent="0.25">
       <c r="A25" s="7">
         <v>24</v>
       </c>
@@ -1597,8 +1677,11 @@
       <c r="C25" s="3" t="s">
         <v>250</v>
       </c>
-    </row>
-    <row r="26" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="D25" s="9"/>
+      <c r="E25" s="9"/>
+      <c r="F25" s="9"/>
+    </row>
+    <row r="26" spans="1:6" ht="16.5" x14ac:dyDescent="0.25">
       <c r="A26" s="7">
         <v>25</v>
       </c>
@@ -1608,8 +1691,11 @@
       <c r="C26" s="3" t="s">
         <v>225</v>
       </c>
-    </row>
-    <row r="27" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="D26" s="9"/>
+      <c r="E26" s="9"/>
+      <c r="F26" s="9"/>
+    </row>
+    <row r="27" spans="1:6" ht="16.5" x14ac:dyDescent="0.25">
       <c r="A27" s="7">
         <v>26</v>
       </c>
@@ -1619,8 +1705,11 @@
       <c r="C27" s="3" t="s">
         <v>262</v>
       </c>
-    </row>
-    <row r="28" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="D27" s="9"/>
+      <c r="E27" s="9"/>
+      <c r="F27" s="9"/>
+    </row>
+    <row r="28" spans="1:6" ht="16.5" x14ac:dyDescent="0.25">
       <c r="A28" s="7">
         <v>27</v>
       </c>
@@ -1630,8 +1719,11 @@
       <c r="C28" s="3" t="s">
         <v>163</v>
       </c>
-    </row>
-    <row r="29" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="D28" s="9"/>
+      <c r="E28" s="9"/>
+      <c r="F28" s="9"/>
+    </row>
+    <row r="29" spans="1:6" ht="16.5" x14ac:dyDescent="0.25">
       <c r="A29" s="7">
         <v>28</v>
       </c>
@@ -1641,8 +1733,11 @@
       <c r="C29" s="3" t="s">
         <v>179</v>
       </c>
-    </row>
-    <row r="30" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="D29" s="9"/>
+      <c r="E29" s="9"/>
+      <c r="F29" s="9"/>
+    </row>
+    <row r="30" spans="1:6" ht="16.5" x14ac:dyDescent="0.25">
       <c r="A30" s="7">
         <v>29</v>
       </c>
@@ -1652,8 +1747,11 @@
       <c r="C30" s="3" t="s">
         <v>226</v>
       </c>
-    </row>
-    <row r="31" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="D30" s="9"/>
+      <c r="E30" s="9"/>
+      <c r="F30" s="9"/>
+    </row>
+    <row r="31" spans="1:6" ht="16.5" x14ac:dyDescent="0.25">
       <c r="A31" s="7">
         <v>30</v>
       </c>
@@ -1663,8 +1761,11 @@
       <c r="C31" s="3" t="s">
         <v>195</v>
       </c>
-    </row>
-    <row r="32" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="D31" s="9"/>
+      <c r="E31" s="9"/>
+      <c r="F31" s="9"/>
+    </row>
+    <row r="32" spans="1:6" ht="16.5" x14ac:dyDescent="0.25">
       <c r="A32" s="7">
         <v>31</v>
       </c>
@@ -1674,8 +1775,11 @@
       <c r="C32" s="3" t="s">
         <v>173</v>
       </c>
-    </row>
-    <row r="33" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="D32" s="9"/>
+      <c r="E32" s="9"/>
+      <c r="F32" s="9"/>
+    </row>
+    <row r="33" spans="1:6" ht="16.5" x14ac:dyDescent="0.25">
       <c r="A33" s="7">
         <v>32</v>
       </c>
@@ -1685,8 +1789,11 @@
       <c r="C33" s="3" t="s">
         <v>187</v>
       </c>
-    </row>
-    <row r="34" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="D33" s="9"/>
+      <c r="E33" s="9"/>
+      <c r="F33" s="9"/>
+    </row>
+    <row r="34" spans="1:6" ht="16.5" x14ac:dyDescent="0.25">
       <c r="A34" s="7">
         <v>33</v>
       </c>
@@ -1696,8 +1803,11 @@
       <c r="C34" s="3" t="s">
         <v>170</v>
       </c>
-    </row>
-    <row r="35" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="D34" s="9"/>
+      <c r="E34" s="9"/>
+      <c r="F34" s="9"/>
+    </row>
+    <row r="35" spans="1:6" ht="16.5" x14ac:dyDescent="0.25">
       <c r="A35" s="7">
         <v>34</v>
       </c>
@@ -1707,8 +1817,11 @@
       <c r="C35" s="3" t="s">
         <v>252</v>
       </c>
-    </row>
-    <row r="36" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="D35" s="9"/>
+      <c r="E35" s="9"/>
+      <c r="F35" s="9"/>
+    </row>
+    <row r="36" spans="1:6" ht="16.5" x14ac:dyDescent="0.25">
       <c r="A36" s="7">
         <v>35</v>
       </c>
@@ -1718,8 +1831,11 @@
       <c r="C36" s="3" t="s">
         <v>258</v>
       </c>
-    </row>
-    <row r="37" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="D36" s="9"/>
+      <c r="E36" s="9"/>
+      <c r="F36" s="9"/>
+    </row>
+    <row r="37" spans="1:6" ht="16.5" x14ac:dyDescent="0.25">
       <c r="A37" s="7">
         <v>36</v>
       </c>
@@ -1729,8 +1845,11 @@
       <c r="C37" s="3" t="s">
         <v>178</v>
       </c>
-    </row>
-    <row r="38" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="D37" s="9"/>
+      <c r="E37" s="9"/>
+      <c r="F37" s="9"/>
+    </row>
+    <row r="38" spans="1:6" ht="16.5" x14ac:dyDescent="0.25">
       <c r="A38" s="7">
         <v>37</v>
       </c>
@@ -1740,8 +1859,11 @@
       <c r="C38" s="3" t="s">
         <v>216</v>
       </c>
-    </row>
-    <row r="39" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="D38" s="9"/>
+      <c r="E38" s="9"/>
+      <c r="F38" s="9"/>
+    </row>
+    <row r="39" spans="1:6" ht="16.5" x14ac:dyDescent="0.25">
       <c r="A39" s="7">
         <v>38</v>
       </c>
@@ -1751,8 +1873,11 @@
       <c r="C39" s="3" t="s">
         <v>183</v>
       </c>
-    </row>
-    <row r="40" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="D39" s="9"/>
+      <c r="E39" s="9"/>
+      <c r="F39" s="9"/>
+    </row>
+    <row r="40" spans="1:6" ht="16.5" x14ac:dyDescent="0.25">
       <c r="A40" s="7">
         <v>39</v>
       </c>
@@ -1762,8 +1887,11 @@
       <c r="C40" s="3" t="s">
         <v>193</v>
       </c>
-    </row>
-    <row r="41" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="D40" s="9"/>
+      <c r="E40" s="9"/>
+      <c r="F40" s="9"/>
+    </row>
+    <row r="41" spans="1:6" ht="16.5" x14ac:dyDescent="0.25">
       <c r="A41" s="7">
         <v>40</v>
       </c>
@@ -1773,8 +1901,11 @@
       <c r="C41" s="3" t="s">
         <v>300</v>
       </c>
-    </row>
-    <row r="42" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="D41" s="9"/>
+      <c r="E41" s="9"/>
+      <c r="F41" s="9"/>
+    </row>
+    <row r="42" spans="1:6" ht="16.5" x14ac:dyDescent="0.25">
       <c r="A42" s="7">
         <v>41</v>
       </c>
@@ -1784,8 +1915,11 @@
       <c r="C42" s="3" t="s">
         <v>229</v>
       </c>
-    </row>
-    <row r="43" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="D42" s="9"/>
+      <c r="E42" s="9"/>
+      <c r="F42" s="9"/>
+    </row>
+    <row r="43" spans="1:6" ht="33" x14ac:dyDescent="0.25">
       <c r="A43" s="7">
         <v>42</v>
       </c>
@@ -1795,8 +1929,11 @@
       <c r="C43" s="3" t="s">
         <v>169</v>
       </c>
-    </row>
-    <row r="44" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="D43" s="9"/>
+      <c r="E43" s="9"/>
+      <c r="F43" s="9"/>
+    </row>
+    <row r="44" spans="1:6" ht="16.5" x14ac:dyDescent="0.25">
       <c r="A44" s="7">
         <v>43</v>
       </c>
@@ -1806,8 +1943,11 @@
       <c r="C44" s="3" t="s">
         <v>228</v>
       </c>
-    </row>
-    <row r="45" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="D44" s="9"/>
+      <c r="E44" s="9"/>
+      <c r="F44" s="9"/>
+    </row>
+    <row r="45" spans="1:6" ht="16.5" x14ac:dyDescent="0.25">
       <c r="A45" s="7">
         <v>44</v>
       </c>
@@ -1817,8 +1957,11 @@
       <c r="C45" s="3" t="s">
         <v>259</v>
       </c>
-    </row>
-    <row r="46" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="D45" s="9"/>
+      <c r="E45" s="9"/>
+      <c r="F45" s="9"/>
+    </row>
+    <row r="46" spans="1:6" ht="16.5" x14ac:dyDescent="0.25">
       <c r="A46" s="7">
         <v>45</v>
       </c>
@@ -1828,8 +1971,11 @@
       <c r="C46" s="3" t="s">
         <v>222</v>
       </c>
-    </row>
-    <row r="47" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="D46" s="9"/>
+      <c r="E46" s="9"/>
+      <c r="F46" s="9"/>
+    </row>
+    <row r="47" spans="1:6" ht="16.5" x14ac:dyDescent="0.25">
       <c r="A47" s="7">
         <v>46</v>
       </c>
@@ -1839,8 +1985,11 @@
       <c r="C47" s="3" t="s">
         <v>186</v>
       </c>
-    </row>
-    <row r="48" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="D47" s="9"/>
+      <c r="E47" s="9"/>
+      <c r="F47" s="9"/>
+    </row>
+    <row r="48" spans="1:6" ht="16.5" x14ac:dyDescent="0.25">
       <c r="A48" s="7">
         <v>47</v>
       </c>
@@ -1850,8 +1999,11 @@
       <c r="C48" s="3" t="s">
         <v>201</v>
       </c>
-    </row>
-    <row r="49" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="D48" s="9"/>
+      <c r="E48" s="9"/>
+      <c r="F48" s="9"/>
+    </row>
+    <row r="49" spans="1:6" ht="16.5" x14ac:dyDescent="0.25">
       <c r="A49" s="7">
         <v>48</v>
       </c>
@@ -1861,8 +2013,11 @@
       <c r="C49" s="3" t="s">
         <v>157</v>
       </c>
-    </row>
-    <row r="50" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="D49" s="9"/>
+      <c r="E49" s="9"/>
+      <c r="F49" s="9"/>
+    </row>
+    <row r="50" spans="1:6" ht="16.5" x14ac:dyDescent="0.25">
       <c r="A50" s="7">
         <v>49</v>
       </c>
@@ -1872,8 +2027,11 @@
       <c r="C50" s="3" t="s">
         <v>203</v>
       </c>
-    </row>
-    <row r="51" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="D50" s="9"/>
+      <c r="E50" s="9"/>
+      <c r="F50" s="9"/>
+    </row>
+    <row r="51" spans="1:6" ht="16.5" x14ac:dyDescent="0.25">
       <c r="A51" s="7">
         <v>50</v>
       </c>
@@ -1883,8 +2041,11 @@
       <c r="C51" s="3" t="s">
         <v>256</v>
       </c>
-    </row>
-    <row r="52" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="D51" s="9"/>
+      <c r="E51" s="9"/>
+      <c r="F51" s="9"/>
+    </row>
+    <row r="52" spans="1:6" ht="16.5" x14ac:dyDescent="0.25">
       <c r="A52" s="7">
         <v>51</v>
       </c>
@@ -1894,8 +2055,11 @@
       <c r="C52" s="3" t="s">
         <v>301</v>
       </c>
-    </row>
-    <row r="53" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="D52" s="9"/>
+      <c r="E52" s="9"/>
+      <c r="F52" s="9"/>
+    </row>
+    <row r="53" spans="1:6" ht="16.5" x14ac:dyDescent="0.25">
       <c r="A53" s="7">
         <v>52</v>
       </c>
@@ -1905,8 +2069,11 @@
       <c r="C53" s="3" t="s">
         <v>285</v>
       </c>
-    </row>
-    <row r="54" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="D53" s="9"/>
+      <c r="E53" s="9"/>
+      <c r="F53" s="9"/>
+    </row>
+    <row r="54" spans="1:6" ht="16.5" x14ac:dyDescent="0.25">
       <c r="A54" s="7">
         <v>53</v>
       </c>
@@ -1916,8 +2083,11 @@
       <c r="C54" s="3" t="s">
         <v>260</v>
       </c>
-    </row>
-    <row r="55" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="D54" s="9"/>
+      <c r="E54" s="9"/>
+      <c r="F54" s="9"/>
+    </row>
+    <row r="55" spans="1:6" ht="16.5" x14ac:dyDescent="0.25">
       <c r="A55" s="7">
         <v>54</v>
       </c>
@@ -1927,8 +2097,11 @@
       <c r="C55" s="3" t="s">
         <v>268</v>
       </c>
-    </row>
-    <row r="56" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="D55" s="9"/>
+      <c r="E55" s="9"/>
+      <c r="F55" s="9"/>
+    </row>
+    <row r="56" spans="1:6" ht="16.5" x14ac:dyDescent="0.25">
       <c r="A56" s="7">
         <v>55</v>
       </c>
@@ -1938,8 +2111,11 @@
       <c r="C56" s="3" t="s">
         <v>206</v>
       </c>
-    </row>
-    <row r="57" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="D56" s="9"/>
+      <c r="E56" s="9"/>
+      <c r="F56" s="9"/>
+    </row>
+    <row r="57" spans="1:6" ht="16.5" x14ac:dyDescent="0.25">
       <c r="A57" s="7">
         <v>56</v>
       </c>
@@ -1949,8 +2125,11 @@
       <c r="C57" s="3" t="s">
         <v>158</v>
       </c>
-    </row>
-    <row r="58" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="D57" s="9"/>
+      <c r="E57" s="9"/>
+      <c r="F57" s="9"/>
+    </row>
+    <row r="58" spans="1:6" ht="16.5" x14ac:dyDescent="0.25">
       <c r="A58" s="7">
         <v>57</v>
       </c>
@@ -1960,8 +2139,11 @@
       <c r="C58" s="3" t="s">
         <v>218</v>
       </c>
-    </row>
-    <row r="59" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="D58" s="9"/>
+      <c r="E58" s="9"/>
+      <c r="F58" s="9"/>
+    </row>
+    <row r="59" spans="1:6" ht="16.5" x14ac:dyDescent="0.25">
       <c r="A59" s="7">
         <v>58</v>
       </c>
@@ -1971,8 +2153,11 @@
       <c r="C59" s="3" t="s">
         <v>239</v>
       </c>
-    </row>
-    <row r="60" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="D59" s="9"/>
+      <c r="E59" s="9"/>
+      <c r="F59" s="9"/>
+    </row>
+    <row r="60" spans="1:6" ht="16.5" x14ac:dyDescent="0.25">
       <c r="A60" s="7">
         <v>59</v>
       </c>
@@ -1982,8 +2167,11 @@
       <c r="C60" s="3" t="s">
         <v>221</v>
       </c>
-    </row>
-    <row r="61" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="D60" s="9"/>
+      <c r="E60" s="9"/>
+      <c r="F60" s="9"/>
+    </row>
+    <row r="61" spans="1:6" ht="16.5" x14ac:dyDescent="0.25">
       <c r="A61" s="7">
         <v>60</v>
       </c>
@@ -1993,8 +2181,11 @@
       <c r="C61" s="3" t="s">
         <v>172</v>
       </c>
-    </row>
-    <row r="62" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="D61" s="9"/>
+      <c r="E61" s="9"/>
+      <c r="F61" s="9"/>
+    </row>
+    <row r="62" spans="1:6" ht="16.5" x14ac:dyDescent="0.25">
       <c r="A62" s="7">
         <v>61</v>
       </c>
@@ -2004,8 +2195,11 @@
       <c r="C62" s="3" t="s">
         <v>273</v>
       </c>
-    </row>
-    <row r="63" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="D62" s="9"/>
+      <c r="E62" s="9"/>
+      <c r="F62" s="9"/>
+    </row>
+    <row r="63" spans="1:6" ht="16.5" x14ac:dyDescent="0.25">
       <c r="A63" s="7">
         <v>62</v>
       </c>
@@ -2015,8 +2209,11 @@
       <c r="C63" s="3" t="s">
         <v>208</v>
       </c>
-    </row>
-    <row r="64" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="D63" s="9"/>
+      <c r="E63" s="9"/>
+      <c r="F63" s="9"/>
+    </row>
+    <row r="64" spans="1:6" ht="16.5" x14ac:dyDescent="0.25">
       <c r="A64" s="7">
         <v>63</v>
       </c>
@@ -2026,8 +2223,11 @@
       <c r="C64" s="3" t="s">
         <v>271</v>
       </c>
-    </row>
-    <row r="65" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="D64" s="9"/>
+      <c r="E64" s="9"/>
+      <c r="F64" s="9"/>
+    </row>
+    <row r="65" spans="1:6" ht="16.5" x14ac:dyDescent="0.25">
       <c r="A65" s="7">
         <v>64</v>
       </c>
@@ -2037,8 +2237,11 @@
       <c r="C65" s="3" t="s">
         <v>274</v>
       </c>
-    </row>
-    <row r="66" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="D65" s="9"/>
+      <c r="E65" s="9"/>
+      <c r="F65" s="9"/>
+    </row>
+    <row r="66" spans="1:6" ht="16.5" x14ac:dyDescent="0.25">
       <c r="A66" s="7">
         <v>65</v>
       </c>
@@ -2048,8 +2251,11 @@
       <c r="C66" s="3" t="s">
         <v>276</v>
       </c>
-    </row>
-    <row r="67" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="D66" s="9"/>
+      <c r="E66" s="9"/>
+      <c r="F66" s="9"/>
+    </row>
+    <row r="67" spans="1:6" ht="16.5" x14ac:dyDescent="0.25">
       <c r="A67" s="7">
         <v>66</v>
       </c>
@@ -2059,8 +2265,11 @@
       <c r="C67" s="3" t="s">
         <v>205</v>
       </c>
-    </row>
-    <row r="68" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="D67" s="9"/>
+      <c r="E67" s="9"/>
+      <c r="F67" s="9"/>
+    </row>
+    <row r="68" spans="1:6" ht="16.5" x14ac:dyDescent="0.25">
       <c r="A68" s="7">
         <v>67</v>
       </c>
@@ -2070,8 +2279,11 @@
       <c r="C68" s="3" t="s">
         <v>213</v>
       </c>
-    </row>
-    <row r="69" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="D68" s="9"/>
+      <c r="E68" s="9"/>
+      <c r="F68" s="9"/>
+    </row>
+    <row r="69" spans="1:6" ht="16.5" x14ac:dyDescent="0.25">
       <c r="A69" s="7">
         <v>68</v>
       </c>
@@ -2081,8 +2293,11 @@
       <c r="C69" s="3" t="s">
         <v>280</v>
       </c>
-    </row>
-    <row r="70" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="D69" s="9"/>
+      <c r="E69" s="9"/>
+      <c r="F69" s="9"/>
+    </row>
+    <row r="70" spans="1:6" ht="33" x14ac:dyDescent="0.25">
       <c r="A70" s="7">
         <v>69</v>
       </c>
@@ -2092,8 +2307,11 @@
       <c r="C70" s="3" t="s">
         <v>257</v>
       </c>
-    </row>
-    <row r="71" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="D70" s="9"/>
+      <c r="E70" s="9"/>
+      <c r="F70" s="9"/>
+    </row>
+    <row r="71" spans="1:6" ht="16.5" x14ac:dyDescent="0.25">
       <c r="A71" s="7">
         <v>70</v>
       </c>
@@ -2103,8 +2321,11 @@
       <c r="C71" s="3" t="s">
         <v>281</v>
       </c>
-    </row>
-    <row r="72" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="D71" s="9"/>
+      <c r="E71" s="9"/>
+      <c r="F71" s="9"/>
+    </row>
+    <row r="72" spans="1:6" ht="33" x14ac:dyDescent="0.25">
       <c r="A72" s="7">
         <v>71</v>
       </c>
@@ -2114,8 +2335,11 @@
       <c r="C72" s="3" t="s">
         <v>248</v>
       </c>
-    </row>
-    <row r="73" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="D72" s="9"/>
+      <c r="E72" s="9"/>
+      <c r="F72" s="9"/>
+    </row>
+    <row r="73" spans="1:6" ht="16.5" x14ac:dyDescent="0.25">
       <c r="A73" s="7">
         <v>72</v>
       </c>
@@ -2125,8 +2349,11 @@
       <c r="C73" s="3" t="s">
         <v>261</v>
       </c>
-    </row>
-    <row r="74" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="D73" s="9"/>
+      <c r="E73" s="9"/>
+      <c r="F73" s="9"/>
+    </row>
+    <row r="74" spans="1:6" ht="16.5" x14ac:dyDescent="0.25">
       <c r="A74" s="7">
         <v>73</v>
       </c>
@@ -2136,8 +2363,11 @@
       <c r="C74" s="3" t="s">
         <v>307</v>
       </c>
-    </row>
-    <row r="75" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="D74" s="9"/>
+      <c r="E74" s="9"/>
+      <c r="F74" s="9"/>
+    </row>
+    <row r="75" spans="1:6" ht="16.5" x14ac:dyDescent="0.25">
       <c r="A75" s="7">
         <v>74</v>
       </c>
@@ -2147,8 +2377,11 @@
       <c r="C75" s="3" t="s">
         <v>263</v>
       </c>
-    </row>
-    <row r="76" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="D75" s="9"/>
+      <c r="E75" s="9"/>
+      <c r="F75" s="9"/>
+    </row>
+    <row r="76" spans="1:6" ht="16.5" x14ac:dyDescent="0.25">
       <c r="A76" s="7">
         <v>75</v>
       </c>
@@ -2158,8 +2391,11 @@
       <c r="C76" s="3" t="s">
         <v>241</v>
       </c>
-    </row>
-    <row r="77" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="D76" s="9"/>
+      <c r="E76" s="9"/>
+      <c r="F76" s="9"/>
+    </row>
+    <row r="77" spans="1:6" ht="16.5" x14ac:dyDescent="0.25">
       <c r="A77" s="7">
         <v>76</v>
       </c>
@@ -2169,8 +2405,11 @@
       <c r="C77" s="3" t="s">
         <v>264</v>
       </c>
-    </row>
-    <row r="78" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="D77" s="9"/>
+      <c r="E77" s="9"/>
+      <c r="F77" s="9"/>
+    </row>
+    <row r="78" spans="1:6" ht="16.5" x14ac:dyDescent="0.25">
       <c r="A78" s="7">
         <v>77</v>
       </c>
@@ -2180,8 +2419,11 @@
       <c r="C78" s="3" t="s">
         <v>290</v>
       </c>
-    </row>
-    <row r="79" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="D78" s="9"/>
+      <c r="E78" s="9"/>
+      <c r="F78" s="9"/>
+    </row>
+    <row r="79" spans="1:6" ht="16.5" x14ac:dyDescent="0.25">
       <c r="A79" s="7">
         <v>78</v>
       </c>
@@ -2191,8 +2433,11 @@
       <c r="C79" s="3" t="s">
         <v>277</v>
       </c>
-    </row>
-    <row r="80" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="D79" s="9"/>
+      <c r="E79" s="9"/>
+      <c r="F79" s="9"/>
+    </row>
+    <row r="80" spans="1:6" ht="16.5" x14ac:dyDescent="0.25">
       <c r="A80" s="7">
         <v>79</v>
       </c>
@@ -2202,8 +2447,11 @@
       <c r="C80" s="3" t="s">
         <v>294</v>
       </c>
-    </row>
-    <row r="81" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="D80" s="9"/>
+      <c r="E80" s="9"/>
+      <c r="F80" s="9"/>
+    </row>
+    <row r="81" spans="1:6" ht="16.5" x14ac:dyDescent="0.25">
       <c r="A81" s="7">
         <v>80</v>
       </c>
@@ -2213,8 +2461,11 @@
       <c r="C81" s="3" t="s">
         <v>185</v>
       </c>
-    </row>
-    <row r="82" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="D81" s="9"/>
+      <c r="E81" s="9"/>
+      <c r="F81" s="9"/>
+    </row>
+    <row r="82" spans="1:6" ht="16.5" x14ac:dyDescent="0.25">
       <c r="A82" s="7">
         <v>81</v>
       </c>
@@ -2224,8 +2475,11 @@
       <c r="C82" s="3" t="s">
         <v>164</v>
       </c>
-    </row>
-    <row r="83" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="D82" s="9"/>
+      <c r="E82" s="9"/>
+      <c r="F82" s="9"/>
+    </row>
+    <row r="83" spans="1:6" ht="16.5" x14ac:dyDescent="0.25">
       <c r="A83" s="7">
         <v>82</v>
       </c>
@@ -2235,8 +2489,11 @@
       <c r="C83" s="3" t="s">
         <v>162</v>
       </c>
-    </row>
-    <row r="84" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="D83" s="9"/>
+      <c r="E83" s="9"/>
+      <c r="F83" s="9"/>
+    </row>
+    <row r="84" spans="1:6" ht="16.5" x14ac:dyDescent="0.25">
       <c r="A84" s="7">
         <v>83</v>
       </c>
@@ -2246,8 +2503,11 @@
       <c r="C84" s="3" t="s">
         <v>293</v>
       </c>
-    </row>
-    <row r="85" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="D84" s="9"/>
+      <c r="E84" s="9"/>
+      <c r="F84" s="9"/>
+    </row>
+    <row r="85" spans="1:6" ht="16.5" x14ac:dyDescent="0.25">
       <c r="A85" s="7">
         <v>84</v>
       </c>
@@ -2257,8 +2517,11 @@
       <c r="C85" s="3" t="s">
         <v>298</v>
       </c>
-    </row>
-    <row r="86" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="D85" s="9"/>
+      <c r="E85" s="9"/>
+      <c r="F85" s="9"/>
+    </row>
+    <row r="86" spans="1:6" ht="33" x14ac:dyDescent="0.25">
       <c r="A86" s="7">
         <v>85</v>
       </c>
@@ -2268,8 +2531,11 @@
       <c r="C86" s="3" t="s">
         <v>160</v>
       </c>
-    </row>
-    <row r="87" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="D86" s="9"/>
+      <c r="E86" s="9"/>
+      <c r="F86" s="9"/>
+    </row>
+    <row r="87" spans="1:6" ht="16.5" x14ac:dyDescent="0.25">
       <c r="A87" s="7">
         <v>86</v>
       </c>
@@ -2279,8 +2545,11 @@
       <c r="C87" s="3" t="s">
         <v>168</v>
       </c>
-    </row>
-    <row r="88" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="D87" s="9"/>
+      <c r="E87" s="9"/>
+      <c r="F87" s="9"/>
+    </row>
+    <row r="88" spans="1:6" ht="16.5" x14ac:dyDescent="0.25">
       <c r="A88" s="7">
         <v>87</v>
       </c>
@@ -2290,8 +2559,11 @@
       <c r="C88" s="3" t="s">
         <v>253</v>
       </c>
-    </row>
-    <row r="89" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="D88" s="9"/>
+      <c r="E88" s="9"/>
+      <c r="F88" s="9"/>
+    </row>
+    <row r="89" spans="1:6" ht="16.5" x14ac:dyDescent="0.25">
       <c r="A89" s="7">
         <v>88</v>
       </c>
@@ -2301,8 +2573,11 @@
       <c r="C89" s="3" t="s">
         <v>265</v>
       </c>
-    </row>
-    <row r="90" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="D89" s="9"/>
+      <c r="E89" s="9"/>
+      <c r="F89" s="9"/>
+    </row>
+    <row r="90" spans="1:6" ht="16.5" x14ac:dyDescent="0.25">
       <c r="A90" s="7">
         <v>89</v>
       </c>
@@ -2312,8 +2587,11 @@
       <c r="C90" s="3" t="s">
         <v>223</v>
       </c>
-    </row>
-    <row r="91" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="D90" s="9"/>
+      <c r="E90" s="9"/>
+      <c r="F90" s="9"/>
+    </row>
+    <row r="91" spans="1:6" ht="16.5" x14ac:dyDescent="0.25">
       <c r="A91" s="7">
         <v>90</v>
       </c>
@@ -2323,8 +2601,11 @@
       <c r="C91" s="3" t="s">
         <v>211</v>
       </c>
-    </row>
-    <row r="92" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="D91" s="9"/>
+      <c r="E91" s="9"/>
+      <c r="F91" s="9"/>
+    </row>
+    <row r="92" spans="1:6" ht="16.5" x14ac:dyDescent="0.25">
       <c r="A92" s="7">
         <v>91</v>
       </c>
@@ -2334,8 +2615,11 @@
       <c r="C92" s="3" t="s">
         <v>215</v>
       </c>
-    </row>
-    <row r="93" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="D92" s="9"/>
+      <c r="E92" s="9"/>
+      <c r="F92" s="9"/>
+    </row>
+    <row r="93" spans="1:6" ht="16.5" x14ac:dyDescent="0.25">
       <c r="A93" s="7">
         <v>92</v>
       </c>
@@ -2345,8 +2629,11 @@
       <c r="C93" s="3" t="s">
         <v>224</v>
       </c>
-    </row>
-    <row r="94" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="D93" s="9"/>
+      <c r="E93" s="9"/>
+      <c r="F93" s="9"/>
+    </row>
+    <row r="94" spans="1:6" ht="16.5" x14ac:dyDescent="0.25">
       <c r="A94" s="7">
         <v>93</v>
       </c>
@@ -2356,8 +2643,11 @@
       <c r="C94" s="3" t="s">
         <v>227</v>
       </c>
-    </row>
-    <row r="95" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="D94" s="9"/>
+      <c r="E94" s="9"/>
+      <c r="F94" s="9"/>
+    </row>
+    <row r="95" spans="1:6" ht="33" x14ac:dyDescent="0.25">
       <c r="A95" s="7">
         <v>94</v>
       </c>
@@ -2367,8 +2657,11 @@
       <c r="C95" s="3" t="s">
         <v>230</v>
       </c>
-    </row>
-    <row r="96" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="D95" s="9"/>
+      <c r="E95" s="9"/>
+      <c r="F95" s="9"/>
+    </row>
+    <row r="96" spans="1:6" ht="16.5" x14ac:dyDescent="0.25">
       <c r="A96" s="7">
         <v>95</v>
       </c>
@@ -2378,8 +2671,11 @@
       <c r="C96" s="3" t="s">
         <v>240</v>
       </c>
-    </row>
-    <row r="97" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="D96" s="9"/>
+      <c r="E96" s="9"/>
+      <c r="F96" s="9"/>
+    </row>
+    <row r="97" spans="1:6" ht="16.5" x14ac:dyDescent="0.25">
       <c r="A97" s="7">
         <v>96</v>
       </c>
@@ -2389,8 +2685,11 @@
       <c r="C97" s="3" t="s">
         <v>190</v>
       </c>
-    </row>
-    <row r="98" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="D97" s="9"/>
+      <c r="E97" s="9"/>
+      <c r="F97" s="9"/>
+    </row>
+    <row r="98" spans="1:6" ht="16.5" x14ac:dyDescent="0.25">
       <c r="A98" s="7">
         <v>97</v>
       </c>
@@ -2400,8 +2699,11 @@
       <c r="C98" s="3" t="s">
         <v>214</v>
       </c>
-    </row>
-    <row r="99" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="D98" s="9"/>
+      <c r="E98" s="9"/>
+      <c r="F98" s="9"/>
+    </row>
+    <row r="99" spans="1:6" ht="16.5" x14ac:dyDescent="0.25">
       <c r="A99" s="7">
         <v>98</v>
       </c>
@@ -2411,8 +2713,11 @@
       <c r="C99" s="3" t="s">
         <v>302</v>
       </c>
-    </row>
-    <row r="100" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="D99" s="9"/>
+      <c r="E99" s="9"/>
+      <c r="F99" s="9"/>
+    </row>
+    <row r="100" spans="1:6" ht="16.5" x14ac:dyDescent="0.25">
       <c r="A100" s="7">
         <v>99</v>
       </c>
@@ -2422,8 +2727,11 @@
       <c r="C100" s="3" t="s">
         <v>279</v>
       </c>
-    </row>
-    <row r="101" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="D100" s="9"/>
+      <c r="E100" s="9"/>
+      <c r="F100" s="9"/>
+    </row>
+    <row r="101" spans="1:6" ht="16.5" x14ac:dyDescent="0.25">
       <c r="A101" s="7">
         <v>100</v>
       </c>
@@ -2433,8 +2741,11 @@
       <c r="C101" s="3" t="s">
         <v>278</v>
       </c>
-    </row>
-    <row r="102" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="D101" s="9"/>
+      <c r="E101" s="9"/>
+      <c r="F101" s="9"/>
+    </row>
+    <row r="102" spans="1:6" ht="16.5" x14ac:dyDescent="0.25">
       <c r="A102" s="7">
         <v>101</v>
       </c>
@@ -2444,8 +2755,11 @@
       <c r="C102" s="3" t="s">
         <v>254</v>
       </c>
-    </row>
-    <row r="103" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="D102" s="9"/>
+      <c r="E102" s="9"/>
+      <c r="F102" s="9"/>
+    </row>
+    <row r="103" spans="1:6" ht="16.5" x14ac:dyDescent="0.25">
       <c r="A103" s="7">
         <v>102</v>
       </c>
@@ -2455,8 +2769,11 @@
       <c r="C103" s="3" t="s">
         <v>204</v>
       </c>
-    </row>
-    <row r="104" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="D103" s="9"/>
+      <c r="E103" s="9"/>
+      <c r="F103" s="9"/>
+    </row>
+    <row r="104" spans="1:6" ht="16.5" x14ac:dyDescent="0.25">
       <c r="A104" s="7">
         <v>103</v>
       </c>
@@ -2466,8 +2783,11 @@
       <c r="C104" s="3" t="s">
         <v>174</v>
       </c>
-    </row>
-    <row r="105" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="D104" s="9"/>
+      <c r="E104" s="9"/>
+      <c r="F104" s="9"/>
+    </row>
+    <row r="105" spans="1:6" ht="16.5" x14ac:dyDescent="0.25">
       <c r="A105" s="7">
         <v>104</v>
       </c>
@@ -2477,8 +2797,11 @@
       <c r="C105" s="3" t="s">
         <v>238</v>
       </c>
-    </row>
-    <row r="106" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="D105" s="9"/>
+      <c r="E105" s="9"/>
+      <c r="F105" s="9"/>
+    </row>
+    <row r="106" spans="1:6" ht="16.5" x14ac:dyDescent="0.25">
       <c r="A106" s="7">
         <v>105</v>
       </c>
@@ -2488,8 +2811,11 @@
       <c r="C106" s="3" t="s">
         <v>220</v>
       </c>
-    </row>
-    <row r="107" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="D106" s="9"/>
+      <c r="E106" s="9"/>
+      <c r="F106" s="9"/>
+    </row>
+    <row r="107" spans="1:6" ht="16.5" x14ac:dyDescent="0.25">
       <c r="A107" s="7">
         <v>106</v>
       </c>
@@ -2499,8 +2825,11 @@
       <c r="C107" s="3" t="s">
         <v>167</v>
       </c>
-    </row>
-    <row r="108" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="D107" s="9"/>
+      <c r="E107" s="9"/>
+      <c r="F107" s="9"/>
+    </row>
+    <row r="108" spans="1:6" ht="16.5" x14ac:dyDescent="0.25">
       <c r="A108" s="7">
         <v>107</v>
       </c>
@@ -2510,8 +2839,11 @@
       <c r="C108" s="3" t="s">
         <v>291</v>
       </c>
-    </row>
-    <row r="109" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="D108" s="9"/>
+      <c r="E108" s="9"/>
+      <c r="F108" s="9"/>
+    </row>
+    <row r="109" spans="1:6" ht="16.5" x14ac:dyDescent="0.25">
       <c r="A109" s="7">
         <v>108</v>
       </c>
@@ -2521,8 +2853,11 @@
       <c r="C109" s="3" t="s">
         <v>197</v>
       </c>
-    </row>
-    <row r="110" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="D109" s="9"/>
+      <c r="E109" s="9"/>
+      <c r="F109" s="9"/>
+    </row>
+    <row r="110" spans="1:6" ht="16.5" x14ac:dyDescent="0.25">
       <c r="A110" s="7">
         <v>109</v>
       </c>
@@ -2532,8 +2867,11 @@
       <c r="C110" s="3" t="s">
         <v>194</v>
       </c>
-    </row>
-    <row r="111" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="D110" s="9"/>
+      <c r="E110" s="9"/>
+      <c r="F110" s="9"/>
+    </row>
+    <row r="111" spans="1:6" ht="16.5" x14ac:dyDescent="0.25">
       <c r="A111" s="7">
         <v>110</v>
       </c>
@@ -2543,8 +2881,11 @@
       <c r="C111" s="3" t="s">
         <v>246</v>
       </c>
-    </row>
-    <row r="112" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="D111" s="9"/>
+      <c r="E111" s="9"/>
+      <c r="F111" s="9"/>
+    </row>
+    <row r="112" spans="1:6" ht="16.5" x14ac:dyDescent="0.25">
       <c r="A112" s="7">
         <v>111</v>
       </c>
@@ -2554,8 +2895,11 @@
       <c r="C112" s="3" t="s">
         <v>303</v>
       </c>
-    </row>
-    <row r="113" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="D112" s="9"/>
+      <c r="E112" s="9"/>
+      <c r="F112" s="9"/>
+    </row>
+    <row r="113" spans="1:6" ht="16.5" x14ac:dyDescent="0.25">
       <c r="A113" s="7">
         <v>112</v>
       </c>
@@ -2565,8 +2909,11 @@
       <c r="C113" s="3" t="s">
         <v>232</v>
       </c>
-    </row>
-    <row r="114" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="D113" s="9"/>
+      <c r="E113" s="9"/>
+      <c r="F113" s="9"/>
+    </row>
+    <row r="114" spans="1:6" ht="16.5" x14ac:dyDescent="0.25">
       <c r="A114" s="7">
         <v>113</v>
       </c>
@@ -2576,8 +2923,11 @@
       <c r="C114" s="3" t="s">
         <v>191</v>
       </c>
-    </row>
-    <row r="115" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="D114" s="9"/>
+      <c r="E114" s="9"/>
+      <c r="F114" s="9"/>
+    </row>
+    <row r="115" spans="1:6" ht="16.5" x14ac:dyDescent="0.25">
       <c r="A115" s="7">
         <v>114</v>
       </c>
@@ -2587,8 +2937,11 @@
       <c r="C115" s="3" t="s">
         <v>287</v>
       </c>
-    </row>
-    <row r="116" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="D115" s="9"/>
+      <c r="E115" s="9"/>
+      <c r="F115" s="9"/>
+    </row>
+    <row r="116" spans="1:6" ht="16.5" x14ac:dyDescent="0.25">
       <c r="A116" s="7">
         <v>115</v>
       </c>
@@ -2598,8 +2951,11 @@
       <c r="C116" s="3" t="s">
         <v>249</v>
       </c>
-    </row>
-    <row r="117" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="D116" s="9"/>
+      <c r="E116" s="9"/>
+      <c r="F116" s="9"/>
+    </row>
+    <row r="117" spans="1:6" ht="16.5" x14ac:dyDescent="0.25">
       <c r="A117" s="7">
         <v>116</v>
       </c>
@@ -2609,8 +2965,11 @@
       <c r="C117" s="3" t="s">
         <v>266</v>
       </c>
-    </row>
-    <row r="118" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="D117" s="9"/>
+      <c r="E117" s="9"/>
+      <c r="F117" s="9"/>
+    </row>
+    <row r="118" spans="1:6" ht="33" x14ac:dyDescent="0.25">
       <c r="A118" s="7">
         <v>117</v>
       </c>
@@ -2620,8 +2979,11 @@
       <c r="C118" s="3" t="s">
         <v>210</v>
       </c>
-    </row>
-    <row r="119" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="D118" s="9"/>
+      <c r="E118" s="9"/>
+      <c r="F118" s="9"/>
+    </row>
+    <row r="119" spans="1:6" ht="16.5" x14ac:dyDescent="0.25">
       <c r="A119" s="7">
         <v>118</v>
       </c>
@@ -2631,8 +2993,11 @@
       <c r="C119" s="3" t="s">
         <v>219</v>
       </c>
-    </row>
-    <row r="120" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="D119" s="9"/>
+      <c r="E119" s="9"/>
+      <c r="F119" s="9"/>
+    </row>
+    <row r="120" spans="1:6" ht="16.5" x14ac:dyDescent="0.25">
       <c r="A120" s="7">
         <v>119</v>
       </c>
@@ -2642,8 +3007,11 @@
       <c r="C120" s="3" t="s">
         <v>188</v>
       </c>
-    </row>
-    <row r="121" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="D120" s="9"/>
+      <c r="E120" s="9"/>
+      <c r="F120" s="9"/>
+    </row>
+    <row r="121" spans="1:6" ht="16.5" x14ac:dyDescent="0.25">
       <c r="A121" s="7">
         <v>120</v>
       </c>
@@ -2653,8 +3021,11 @@
       <c r="C121" s="3" t="s">
         <v>255</v>
       </c>
-    </row>
-    <row r="122" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="D121" s="9"/>
+      <c r="E121" s="9"/>
+      <c r="F121" s="9"/>
+    </row>
+    <row r="122" spans="1:6" ht="16.5" x14ac:dyDescent="0.25">
       <c r="A122" s="7">
         <v>121</v>
       </c>
@@ -2664,8 +3035,11 @@
       <c r="C122" s="3" t="s">
         <v>282</v>
       </c>
-    </row>
-    <row r="123" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="D122" s="9"/>
+      <c r="E122" s="9"/>
+      <c r="F122" s="9"/>
+    </row>
+    <row r="123" spans="1:6" ht="16.5" x14ac:dyDescent="0.25">
       <c r="A123" s="7">
         <v>122</v>
       </c>
@@ -2675,8 +3049,11 @@
       <c r="C123" s="3" t="s">
         <v>165</v>
       </c>
-    </row>
-    <row r="124" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="D123" s="9"/>
+      <c r="E123" s="9"/>
+      <c r="F123" s="9"/>
+    </row>
+    <row r="124" spans="1:6" ht="16.5" x14ac:dyDescent="0.25">
       <c r="A124" s="7">
         <v>123</v>
       </c>
@@ -2686,8 +3063,11 @@
       <c r="C124" s="3" t="s">
         <v>288</v>
       </c>
-    </row>
-    <row r="125" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="D124" s="9"/>
+      <c r="E124" s="9"/>
+      <c r="F124" s="9"/>
+    </row>
+    <row r="125" spans="1:6" ht="16.5" x14ac:dyDescent="0.25">
       <c r="A125" s="7">
         <v>124</v>
       </c>
@@ -2697,8 +3077,11 @@
       <c r="C125" s="3" t="s">
         <v>196</v>
       </c>
-    </row>
-    <row r="126" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="D125" s="9"/>
+      <c r="E125" s="9"/>
+      <c r="F125" s="9"/>
+    </row>
+    <row r="126" spans="1:6" ht="16.5" x14ac:dyDescent="0.25">
       <c r="A126" s="7">
         <v>125</v>
       </c>
@@ -2708,8 +3091,11 @@
       <c r="C126" s="3" t="s">
         <v>189</v>
       </c>
-    </row>
-    <row r="127" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="D126" s="9"/>
+      <c r="E126" s="9"/>
+      <c r="F126" s="9"/>
+    </row>
+    <row r="127" spans="1:6" ht="16.5" x14ac:dyDescent="0.25">
       <c r="A127" s="7">
         <v>126</v>
       </c>
@@ -2719,8 +3105,11 @@
       <c r="C127" s="3" t="s">
         <v>182</v>
       </c>
-    </row>
-    <row r="128" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="D127" s="9"/>
+      <c r="E127" s="9"/>
+      <c r="F127" s="9"/>
+    </row>
+    <row r="128" spans="1:6" ht="16.5" x14ac:dyDescent="0.25">
       <c r="A128" s="7">
         <v>127</v>
       </c>
@@ -2730,8 +3119,11 @@
       <c r="C128" s="3" t="s">
         <v>199</v>
       </c>
-    </row>
-    <row r="129" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="D128" s="9"/>
+      <c r="E128" s="9"/>
+      <c r="F128" s="9"/>
+    </row>
+    <row r="129" spans="1:6" ht="16.5" x14ac:dyDescent="0.25">
       <c r="A129" s="7">
         <v>128</v>
       </c>
@@ -2741,8 +3133,11 @@
       <c r="C129" s="3" t="s">
         <v>292</v>
       </c>
-    </row>
-    <row r="130" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="D129" s="9"/>
+      <c r="E129" s="9"/>
+      <c r="F129" s="9"/>
+    </row>
+    <row r="130" spans="1:6" ht="16.5" x14ac:dyDescent="0.25">
       <c r="A130" s="7">
         <v>129</v>
       </c>
@@ -2752,8 +3147,11 @@
       <c r="C130" s="3" t="s">
         <v>283</v>
       </c>
-    </row>
-    <row r="131" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="D130" s="9"/>
+      <c r="E130" s="9"/>
+      <c r="F130" s="9"/>
+    </row>
+    <row r="131" spans="1:6" ht="16.5" x14ac:dyDescent="0.25">
       <c r="A131" s="7">
         <v>130</v>
       </c>
@@ -2763,8 +3161,11 @@
       <c r="C131" s="3" t="s">
         <v>192</v>
       </c>
-    </row>
-    <row r="132" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="D131" s="9"/>
+      <c r="E131" s="9"/>
+      <c r="F131" s="9"/>
+    </row>
+    <row r="132" spans="1:6" ht="16.5" x14ac:dyDescent="0.25">
       <c r="A132" s="7">
         <v>131</v>
       </c>
@@ -2774,8 +3175,11 @@
       <c r="C132" s="3" t="s">
         <v>289</v>
       </c>
-    </row>
-    <row r="133" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="D132" s="9"/>
+      <c r="E132" s="9"/>
+      <c r="F132" s="9"/>
+    </row>
+    <row r="133" spans="1:6" ht="16.5" x14ac:dyDescent="0.25">
       <c r="A133" s="7">
         <v>132</v>
       </c>
@@ -2785,8 +3189,11 @@
       <c r="C133" s="3" t="s">
         <v>234</v>
       </c>
-    </row>
-    <row r="134" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="D133" s="9"/>
+      <c r="E133" s="9"/>
+      <c r="F133" s="9"/>
+    </row>
+    <row r="134" spans="1:6" ht="16.5" x14ac:dyDescent="0.25">
       <c r="A134" s="7">
         <v>133</v>
       </c>
@@ -2796,8 +3203,11 @@
       <c r="C134" s="3" t="s">
         <v>181</v>
       </c>
-    </row>
-    <row r="135" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="D134" s="9"/>
+      <c r="E134" s="9"/>
+      <c r="F134" s="9"/>
+    </row>
+    <row r="135" spans="1:6" ht="16.5" x14ac:dyDescent="0.25">
       <c r="A135" s="7">
         <v>134</v>
       </c>
@@ -2807,8 +3217,11 @@
       <c r="C135" s="3" t="s">
         <v>233</v>
       </c>
-    </row>
-    <row r="136" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="D135" s="9"/>
+      <c r="E135" s="9"/>
+      <c r="F135" s="9"/>
+    </row>
+    <row r="136" spans="1:6" ht="16.5" x14ac:dyDescent="0.25">
       <c r="A136" s="7">
         <v>135</v>
       </c>
@@ -2818,8 +3231,11 @@
       <c r="C136" s="3" t="s">
         <v>235</v>
       </c>
-    </row>
-    <row r="137" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="D136" s="9"/>
+      <c r="E136" s="9"/>
+      <c r="F136" s="9"/>
+    </row>
+    <row r="137" spans="1:6" ht="16.5" x14ac:dyDescent="0.25">
       <c r="A137" s="7">
         <v>136</v>
       </c>
@@ -2829,8 +3245,11 @@
       <c r="C137" s="3" t="s">
         <v>296</v>
       </c>
-    </row>
-    <row r="138" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="D137" s="9"/>
+      <c r="E137" s="9"/>
+      <c r="F137" s="9"/>
+    </row>
+    <row r="138" spans="1:6" ht="16.5" x14ac:dyDescent="0.25">
       <c r="A138" s="7">
         <v>137</v>
       </c>
@@ -2840,8 +3259,11 @@
       <c r="C138" s="3" t="s">
         <v>236</v>
       </c>
-    </row>
-    <row r="139" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="D138" s="9"/>
+      <c r="E138" s="9"/>
+      <c r="F138" s="9"/>
+    </row>
+    <row r="139" spans="1:6" ht="16.5" x14ac:dyDescent="0.25">
       <c r="A139" s="7">
         <v>138</v>
       </c>
@@ -2851,8 +3273,11 @@
       <c r="C139" s="3" t="s">
         <v>231</v>
       </c>
-    </row>
-    <row r="140" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="D139" s="9"/>
+      <c r="E139" s="9"/>
+      <c r="F139" s="9"/>
+    </row>
+    <row r="140" spans="1:6" ht="16.5" x14ac:dyDescent="0.25">
       <c r="A140" s="7">
         <v>139</v>
       </c>
@@ -2862,8 +3287,11 @@
       <c r="C140" s="3" t="s">
         <v>297</v>
       </c>
-    </row>
-    <row r="141" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="D140" s="9"/>
+      <c r="E140" s="9"/>
+      <c r="F140" s="9"/>
+    </row>
+    <row r="141" spans="1:6" ht="16.5" x14ac:dyDescent="0.25">
       <c r="A141" s="7">
         <v>140</v>
       </c>
@@ -2873,8 +3301,11 @@
       <c r="C141" s="3" t="s">
         <v>198</v>
       </c>
-    </row>
-    <row r="142" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="D141" s="9"/>
+      <c r="E141" s="9"/>
+      <c r="F141" s="9"/>
+    </row>
+    <row r="142" spans="1:6" ht="16.5" x14ac:dyDescent="0.25">
       <c r="A142" s="7">
         <v>141</v>
       </c>
@@ -2884,8 +3315,11 @@
       <c r="C142" s="3" t="s">
         <v>207</v>
       </c>
-    </row>
-    <row r="143" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="D142" s="9"/>
+      <c r="E142" s="9"/>
+      <c r="F142" s="9"/>
+    </row>
+    <row r="143" spans="1:6" ht="16.5" x14ac:dyDescent="0.25">
       <c r="A143" s="7">
         <v>142</v>
       </c>
@@ -2895,8 +3329,11 @@
       <c r="C143" s="3" t="s">
         <v>299</v>
       </c>
-    </row>
-    <row r="144" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="D143" s="9"/>
+      <c r="E143" s="9"/>
+      <c r="F143" s="9"/>
+    </row>
+    <row r="144" spans="1:6" ht="16.5" x14ac:dyDescent="0.25">
       <c r="A144" s="7">
         <v>143</v>
       </c>
@@ -2906,8 +3343,11 @@
       <c r="C144" s="3" t="s">
         <v>243</v>
       </c>
-    </row>
-    <row r="145" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="D144" s="9"/>
+      <c r="E144" s="9"/>
+      <c r="F144" s="9"/>
+    </row>
+    <row r="145" spans="1:6" ht="16.5" x14ac:dyDescent="0.25">
       <c r="A145" s="7">
         <v>144</v>
       </c>
@@ -2917,8 +3357,11 @@
       <c r="C145" s="3" t="s">
         <v>159</v>
       </c>
-    </row>
-    <row r="146" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="D145" s="9"/>
+      <c r="E145" s="9"/>
+      <c r="F145" s="9"/>
+    </row>
+    <row r="146" spans="1:6" ht="16.5" x14ac:dyDescent="0.25">
       <c r="A146" s="7">
         <v>145</v>
       </c>
@@ -2928,8 +3371,11 @@
       <c r="C146" s="3" t="s">
         <v>212</v>
       </c>
-    </row>
-    <row r="147" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="D146" s="9"/>
+      <c r="E146" s="9"/>
+      <c r="F146" s="9"/>
+    </row>
+    <row r="147" spans="1:6" ht="16.5" x14ac:dyDescent="0.25">
       <c r="A147" s="7">
         <v>146</v>
       </c>
@@ -2939,8 +3385,11 @@
       <c r="C147" s="3" t="s">
         <v>180</v>
       </c>
-    </row>
-    <row r="148" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="D147" s="9"/>
+      <c r="E147" s="9"/>
+      <c r="F147" s="9"/>
+    </row>
+    <row r="148" spans="1:6" ht="16.5" x14ac:dyDescent="0.25">
       <c r="A148" s="7">
         <v>147</v>
       </c>
@@ -2950,8 +3399,11 @@
       <c r="C148" s="3" t="s">
         <v>237</v>
       </c>
-    </row>
-    <row r="149" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="D148" s="9"/>
+      <c r="E148" s="9"/>
+      <c r="F148" s="9"/>
+    </row>
+    <row r="149" spans="1:6" ht="16.5" x14ac:dyDescent="0.25">
       <c r="A149" s="7">
         <v>148</v>
       </c>
@@ -2961,8 +3413,11 @@
       <c r="C149" s="3" t="s">
         <v>217</v>
       </c>
-    </row>
-    <row r="150" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="D149" s="9"/>
+      <c r="E149" s="9"/>
+      <c r="F149" s="9"/>
+    </row>
+    <row r="150" spans="1:6" ht="16.5" x14ac:dyDescent="0.25">
       <c r="A150" s="7">
         <v>149</v>
       </c>
@@ -2972,8 +3427,11 @@
       <c r="C150" s="3" t="s">
         <v>209</v>
       </c>
-    </row>
-    <row r="151" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="D150" s="9"/>
+      <c r="E150" s="9"/>
+      <c r="F150" s="9"/>
+    </row>
+    <row r="151" spans="1:6" ht="16.5" x14ac:dyDescent="0.25">
       <c r="A151" s="7">
         <v>150</v>
       </c>
@@ -2983,8 +3441,11 @@
       <c r="C151" s="3" t="s">
         <v>267</v>
       </c>
-    </row>
-    <row r="152" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="D151" s="9"/>
+      <c r="E151" s="9"/>
+      <c r="F151" s="9"/>
+    </row>
+    <row r="152" spans="1:6" ht="16.5" x14ac:dyDescent="0.25">
       <c r="A152" s="7">
         <v>151</v>
       </c>
@@ -2994,8 +3455,11 @@
       <c r="C152" s="3" t="s">
         <v>202</v>
       </c>
-    </row>
-    <row r="153" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="D152" s="9"/>
+      <c r="E152" s="9"/>
+      <c r="F152" s="9"/>
+    </row>
+    <row r="153" spans="1:6" ht="16.5" x14ac:dyDescent="0.25">
       <c r="A153" s="7">
         <v>152</v>
       </c>
@@ -3005,8 +3469,11 @@
       <c r="C153" s="3" t="s">
         <v>284</v>
       </c>
-    </row>
-    <row r="154" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="D153" s="9"/>
+      <c r="E153" s="9"/>
+      <c r="F153" s="9"/>
+    </row>
+    <row r="154" spans="1:6" ht="16.5" x14ac:dyDescent="0.25">
       <c r="A154" s="7">
         <v>153</v>
       </c>
@@ -3016,6 +3483,9 @@
       <c r="C154" s="3" t="s">
         <v>286</v>
       </c>
+      <c r="D154" s="9"/>
+      <c r="E154" s="9"/>
+      <c r="F154" s="9"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>